<commit_message>
Fix in-game header flicker: the speaker slot borrowed the score block's width (only borrow a sibling button's), fixed right-edge slot, no dock transitions; WebKit+Chromium check with video; roadmap update
</commit_message>
<xml_diff>
--- a/docs/BWM-roadmap.xlsx
+++ b/docs/BWM-roadmap.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="mmm d, yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mmm d, yyyy"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -99,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,7 +115,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -752,7 +754,7 @@
           <t>Rules checked by automated tests and thousands of simulated games</t>
         </is>
       </c>
-      <c r="F2" s="12" t="n">
+      <c r="F2" s="13" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -778,7 +780,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr"/>
-      <c r="F3" s="12" t="n">
+      <c r="F3" s="13" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -804,7 +806,7 @@
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr"/>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="13" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -834,7 +836,7 @@
           <t>3-player game removes a card so the deck divides evenly</t>
         </is>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="13" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -864,7 +866,7 @@
           <t>Bid and play on their own so you can play solo</t>
         </is>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="13" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -894,7 +896,7 @@
           <t>Real 3D table, cards and camera</t>
         </is>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="13" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -920,7 +922,7 @@
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr"/>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="13" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -946,7 +948,7 @@
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr"/>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -976,7 +978,7 @@
           <t>Shuffled, crossfades between tracks; grew to 17 tracks in Release 4, all volume-matched</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F10" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1002,7 +1004,7 @@
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr"/>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1028,7 +1030,7 @@
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr"/>
-      <c r="F12" s="12" t="n">
+      <c r="F12" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1058,7 +1060,7 @@
           <t>Server runs the rules so nobody can cheat; bots fill empty seats; reconnects after drops</t>
         </is>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1088,7 +1090,7 @@
           <t>Optional camera and microphone for each player</t>
         </is>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F14" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1118,7 +1120,7 @@
           <t>Also cut online data use by about 60%</t>
         </is>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1144,7 +1146,7 @@
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr"/>
-      <c r="F16" s="12" t="n">
+      <c r="F16" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1170,7 +1172,7 @@
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr"/>
-      <c r="F17" s="12" t="n">
+      <c r="F17" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1200,7 +1202,7 @@
           <t>Expanded in Releases 3 and 4</t>
         </is>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1226,7 +1228,7 @@
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr"/>
-      <c r="F19" s="12" t="n">
+      <c r="F19" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1256,7 +1258,7 @@
           <t>On by default, can be switched off</t>
         </is>
       </c>
-      <c r="F20" s="12" t="n">
+      <c r="F20" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1282,7 +1284,7 @@
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr"/>
-      <c r="F21" s="12" t="n">
+      <c r="F21" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1308,7 +1310,7 @@
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr"/>
-      <c r="F22" s="12" t="n">
+      <c r="F22" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1334,7 +1336,7 @@
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr"/>
-      <c r="F23" s="12" t="n">
+      <c r="F23" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1364,7 +1366,7 @@
           <t>Host sets the countdown (15 to 45 seconds)</t>
         </is>
       </c>
-      <c r="F24" s="12" t="n">
+      <c r="F24" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1390,7 +1392,7 @@
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr"/>
-      <c r="F25" s="12" t="n">
+      <c r="F25" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1416,7 +1418,7 @@
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr"/>
-      <c r="F26" s="12" t="n">
+      <c r="F26" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1442,7 +1444,7 @@
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr"/>
-      <c r="F27" s="12" t="n">
+      <c r="F27" s="13" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -1472,7 +1474,7 @@
           <t>Off by default; partners can always talk during bidding</t>
         </is>
       </c>
-      <c r="F28" s="12" t="n">
+      <c r="F28" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1498,7 +1500,7 @@
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr"/>
-      <c r="F29" s="12" t="n">
+      <c r="F29" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1528,7 +1530,7 @@
           <t>Tips point at the cards they talk about</t>
         </is>
       </c>
-      <c r="F30" s="12" t="n">
+      <c r="F30" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1554,7 +1556,7 @@
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr"/>
-      <c r="F31" s="12" t="n">
+      <c r="F31" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1580,7 +1582,7 @@
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr"/>
-      <c r="F32" s="12" t="n">
+      <c r="F32" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1610,7 +1612,7 @@
           <t>Includes a private admin page to read feedback</t>
         </is>
       </c>
-      <c r="F33" s="12" t="n">
+      <c r="F33" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1636,7 +1638,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr"/>
-      <c r="F34" s="12" t="n">
+      <c r="F34" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1662,7 +1664,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr"/>
-      <c r="F35" s="12" t="n">
+      <c r="F35" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1688,7 +1690,7 @@
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr"/>
-      <c r="F36" s="12" t="n">
+      <c r="F36" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1718,7 +1720,7 @@
           <t>Host picks intensity: Full Nuke / Classic / Off</t>
         </is>
       </c>
-      <c r="F37" s="12" t="n">
+      <c r="F37" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1748,7 +1750,7 @@
           <t>Expanded to 19 personalities in Release 5</t>
         </is>
       </c>
-      <c r="F38" s="12" t="n">
+      <c r="F38" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1774,7 +1776,7 @@
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr"/>
-      <c r="F39" s="12" t="n">
+      <c r="F39" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1800,7 +1802,7 @@
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr"/>
-      <c r="F40" s="12" t="n">
+      <c r="F40" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1826,7 +1828,7 @@
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr"/>
-      <c r="F41" s="12" t="n">
+      <c r="F41" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1852,7 +1854,7 @@
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr"/>
-      <c r="F42" s="12" t="n">
+      <c r="F42" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1878,7 +1880,7 @@
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr"/>
-      <c r="F43" s="12" t="n">
+      <c r="F43" s="13" t="n">
         <v>46305</v>
       </c>
     </row>
@@ -1908,7 +1910,7 @@
           <t>19 personalities, each in both voices</t>
         </is>
       </c>
-      <c r="F44" s="12" t="n">
+      <c r="F44" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -1938,7 +1940,7 @@
           <t>Smarter bots: count cards, don't waste Jokers, don't trump their partner</t>
         </is>
       </c>
-      <c r="F45" s="12" t="n">
+      <c r="F45" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -1964,7 +1966,7 @@
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr"/>
-      <c r="F46" s="12" t="n">
+      <c r="F46" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -1994,7 +1996,7 @@
           <t>Includes 'Slow your roll, cowboy!'</t>
         </is>
       </c>
-      <c r="F47" s="12" t="n">
+      <c r="F47" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2024,7 +2026,7 @@
           <t>With a first-hand minimum option</t>
         </is>
       </c>
-      <c r="F48" s="12" t="n">
+      <c r="F48" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2054,7 +2056,7 @@
           <t>Pace and social settings can still change</t>
         </is>
       </c>
-      <c r="F49" s="12" t="n">
+      <c r="F49" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2080,7 +2082,7 @@
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr"/>
-      <c r="F50" s="12" t="n">
+      <c r="F50" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2106,7 +2108,7 @@
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr"/>
-      <c r="F51" s="12" t="n">
+      <c r="F51" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2136,7 +2138,7 @@
           <t>Built across Releases 3 to 5</t>
         </is>
       </c>
-      <c r="F52" s="12" t="n">
+      <c r="F52" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2166,7 +2168,7 @@
           <t>Cutthroat still bids clockwise</t>
         </is>
       </c>
-      <c r="F53" s="12" t="n">
+      <c r="F53" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2196,7 +2198,7 @@
           <t>Partner talk presets like '3-ish' and 'I'm weak'; bot partners say their count</t>
         </is>
       </c>
-      <c r="F54" s="12" t="n">
+      <c r="F54" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2222,7 +2224,7 @@
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr"/>
-      <c r="F55" s="12" t="n">
+      <c r="F55" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2252,7 +2254,7 @@
           <t>3-player removes the lowest non-spade card</t>
         </is>
       </c>
-      <c r="F56" s="12" t="n">
+      <c r="F56" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2278,7 +2280,7 @@
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr"/>
-      <c r="F57" s="12" t="n">
+      <c r="F57" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2304,7 +2306,7 @@
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr"/>
-      <c r="F58" s="12" t="n">
+      <c r="F58" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2330,7 +2332,7 @@
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr"/>
-      <c r="F59" s="12" t="n">
+      <c r="F59" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2356,7 +2358,7 @@
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr"/>
-      <c r="F60" s="12" t="n">
+      <c r="F60" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2386,7 +2388,7 @@
           <t>github.com/M33CH1384/bid-wit-me</t>
         </is>
       </c>
-      <c r="F61" s="12" t="n"/>
+      <c r="F61" s="13" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
@@ -2410,7 +2412,7 @@
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr"/>
-      <c r="F62" s="12" t="n">
+      <c r="F62" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2440,7 +2442,7 @@
           <t>Text and recorded clips</t>
         </is>
       </c>
-      <c r="F63" s="12" t="n">
+      <c r="F63" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2466,7 +2468,7 @@
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr"/>
-      <c r="F64" s="12" t="n">
+      <c r="F64" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2492,7 +2494,7 @@
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr"/>
-      <c r="F65" s="12" t="n">
+      <c r="F65" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2522,7 +2524,7 @@
           <t>Also clearer scoreboard on phones and card art fixes</t>
         </is>
       </c>
-      <c r="F66" s="12" t="n">
+      <c r="F66" s="13" t="n">
         <v>46306</v>
       </c>
     </row>
@@ -2552,7 +2554,7 @@
           <t>Work started Oct 11</t>
         </is>
       </c>
-      <c r="F67" s="12" t="n"/>
+      <c r="F67" s="13" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
@@ -2576,7 +2578,7 @@
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr"/>
-      <c r="F68" s="12" t="n"/>
+      <c r="F68" s="13" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
@@ -2604,7 +2606,7 @@
           <t>Plan written: security hardening first, then optional sign-in; guest play stays the default</t>
         </is>
       </c>
-      <c r="F69" s="12" t="n"/>
+      <c r="F69" s="13" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
@@ -2624,7 +2626,7 @@
       </c>
       <c r="D70" s="11" t="inlineStr"/>
       <c r="E70" s="11" t="inlineStr"/>
-      <c r="F70" s="12" t="n"/>
+      <c r="F70" s="13" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="11" t="inlineStr">
@@ -2648,7 +2650,7 @@
           <t>Apple later (needs $99/yr Apple developer account)</t>
         </is>
       </c>
-      <c r="F71" s="12" t="n"/>
+      <c r="F71" s="13" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
@@ -2668,7 +2670,7 @@
       </c>
       <c r="D72" s="11" t="inlineStr"/>
       <c r="E72" s="11" t="inlineStr"/>
-      <c r="F72" s="12" t="n"/>
+      <c r="F72" s="13" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="11" t="inlineStr">
@@ -2688,7 +2690,7 @@
       </c>
       <c r="D73" s="11" t="inlineStr"/>
       <c r="E73" s="11" t="inlineStr"/>
-      <c r="F73" s="12" t="n"/>
+      <c r="F73" s="13" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="11" t="inlineStr">
@@ -2708,7 +2710,7 @@
       </c>
       <c r="D74" s="11" t="inlineStr"/>
       <c r="E74" s="11" t="inlineStr"/>
-      <c r="F74" s="12" t="n"/>
+      <c r="F74" s="13" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="11" t="inlineStr">
@@ -2728,7 +2730,7 @@
       </c>
       <c r="D75" s="11" t="inlineStr"/>
       <c r="E75" s="11" t="inlineStr"/>
-      <c r="F75" s="12" t="n"/>
+      <c r="F75" s="13" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="11" t="inlineStr">
@@ -2748,7 +2750,7 @@
       </c>
       <c r="D76" s="11" t="inlineStr"/>
       <c r="E76" s="11" t="inlineStr"/>
-      <c r="F76" s="12" t="n"/>
+      <c r="F76" s="13" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="11" t="inlineStr">
@@ -2768,7 +2770,7 @@
       </c>
       <c r="D77" s="11" t="inlineStr"/>
       <c r="E77" s="11" t="inlineStr"/>
-      <c r="F77" s="12" t="n"/>
+      <c r="F77" s="13" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="11" t="inlineStr">
@@ -2788,7 +2790,7 @@
       </c>
       <c r="D78" s="11" t="inlineStr"/>
       <c r="E78" s="11" t="inlineStr"/>
-      <c r="F78" s="12" t="n"/>
+      <c r="F78" s="13" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="11" t="inlineStr">
@@ -2812,7 +2814,7 @@
           <t>Storm Chaser already exists on-device</t>
         </is>
       </c>
-      <c r="F79" s="12" t="n"/>
+      <c r="F79" s="13" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
@@ -2832,7 +2834,7 @@
       </c>
       <c r="D80" s="11" t="inlineStr"/>
       <c r="E80" s="11" t="inlineStr"/>
-      <c r="F80" s="12" t="n"/>
+      <c r="F80" s="13" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="11" t="inlineStr">
@@ -2842,7 +2844,7 @@
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Native apps (iPhone / Android)</t>
+          <t>Stretch goal: wrap as native iPhone app (e.g. Capacitor) once core features are stable, to enable iOS haptics and App Store release</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
@@ -2851,8 +2853,12 @@
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr"/>
-      <c r="E81" s="11" t="inlineStr"/>
-      <c r="F81" s="12" t="n"/>
+      <c r="E81" s="11" t="inlineStr">
+        <is>
+          <t>Shared haptic() helper (Android vibration, built by SWE) gets swapped for native haptics in the wrapper</t>
+        </is>
+      </c>
+      <c r="F81" s="13" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F81"/>

</xml_diff>